<commit_message>
montos de 10k en 10k hasta 800k
</commit_message>
<xml_diff>
--- a/grilla.xlsx
+++ b/grilla.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aetch\Desktop\proyecto_aamas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AA50334-2057-454D-B350-F6F49235F240}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34180D95-C8A3-4354-809E-62C986C24B74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1125" yWindow="1125" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Grilla" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="115">
   <si>
     <t>Cuotas12</t>
   </si>
@@ -370,9 +370,6 @@
   </si>
   <si>
     <t>Monto</t>
-  </si>
-  <si>
-    <t>0.00</t>
   </si>
   <si>
     <t>Cuotas6</t>
@@ -388,16 +385,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -425,11 +414,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -782,13 +770,13 @@
         <v>111</v>
       </c>
       <c r="B1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D1" t="s">
         <v>113</v>
-      </c>
-      <c r="D1" t="s">
-        <v>114</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
@@ -804,14 +792,14 @@
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
-        <v>112</v>
-      </c>
-      <c r="C2" t="s">
-        <v>112</v>
-      </c>
-      <c r="D2" t="s">
-        <v>112</v>
+      <c r="B2">
+        <v>11459.35</v>
+      </c>
+      <c r="C2">
+        <v>6200.37</v>
+      </c>
+      <c r="D2">
+        <v>4463.1099999999997</v>
       </c>
       <c r="E2">
         <v>3606.13</v>
@@ -827,14 +815,14 @@
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
-        <v>112</v>
-      </c>
-      <c r="C3" t="s">
-        <v>112</v>
-      </c>
-      <c r="D3" t="s">
-        <v>112</v>
+      <c r="B3">
+        <v>15279.14</v>
+      </c>
+      <c r="C3">
+        <v>8267.16</v>
+      </c>
+      <c r="D3">
+        <v>5950.81</v>
       </c>
       <c r="E3">
         <v>4808.17</v>
@@ -850,14 +838,14 @@
       <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" t="s">
-        <v>112</v>
-      </c>
-      <c r="C4" t="s">
-        <v>112</v>
-      </c>
-      <c r="D4" t="s">
-        <v>112</v>
+      <c r="B4">
+        <v>19098.919999999998</v>
+      </c>
+      <c r="C4">
+        <v>10333.950000000001</v>
+      </c>
+      <c r="D4">
+        <v>7438.52</v>
       </c>
       <c r="E4">
         <v>6010.21</v>
@@ -873,14 +861,14 @@
       <c r="A5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" t="s">
-        <v>112</v>
-      </c>
-      <c r="C5" t="s">
-        <v>112</v>
-      </c>
-      <c r="D5" t="s">
-        <v>112</v>
+      <c r="B5">
+        <v>22918.71</v>
+      </c>
+      <c r="C5">
+        <v>12400.73</v>
+      </c>
+      <c r="D5">
+        <v>8926.2199999999993</v>
       </c>
       <c r="E5">
         <v>7212.25</v>
@@ -896,14 +884,14 @@
       <c r="A6" t="s">
         <v>7</v>
       </c>
-      <c r="B6" t="s">
-        <v>112</v>
-      </c>
-      <c r="C6" t="s">
-        <v>112</v>
-      </c>
-      <c r="D6" t="s">
-        <v>112</v>
+      <c r="B6">
+        <v>26738.49</v>
+      </c>
+      <c r="C6">
+        <v>14467.52</v>
+      </c>
+      <c r="D6">
+        <v>10413.92</v>
       </c>
       <c r="E6">
         <v>8414.2999999999993</v>
@@ -919,14 +907,14 @@
       <c r="A7" t="s">
         <v>8</v>
       </c>
-      <c r="B7" t="s">
-        <v>112</v>
-      </c>
-      <c r="C7" t="s">
-        <v>112</v>
-      </c>
-      <c r="D7" t="s">
-        <v>112</v>
+      <c r="B7">
+        <v>30558.27</v>
+      </c>
+      <c r="C7">
+        <v>16534.310000000001</v>
+      </c>
+      <c r="D7">
+        <v>11901.63</v>
       </c>
       <c r="E7">
         <v>9616.64</v>
@@ -942,14 +930,14 @@
       <c r="A8" t="s">
         <v>9</v>
       </c>
-      <c r="B8" t="s">
-        <v>112</v>
-      </c>
-      <c r="C8" t="s">
-        <v>112</v>
-      </c>
-      <c r="D8" t="s">
-        <v>112</v>
+      <c r="B8">
+        <v>34378.06</v>
+      </c>
+      <c r="C8">
+        <v>18601.099999999999</v>
+      </c>
+      <c r="D8">
+        <v>13389.33</v>
       </c>
       <c r="E8">
         <v>10818.38</v>
@@ -989,13 +977,13 @@
         <v>11</v>
       </c>
       <c r="B10">
-        <v>22734.68</v>
+        <v>42017.63</v>
       </c>
       <c r="C10">
         <v>22734.68</v>
       </c>
-      <c r="D10" t="s">
-        <v>112</v>
+      <c r="D10">
+        <v>16364.74</v>
       </c>
       <c r="E10">
         <v>13222.46</v>
@@ -1011,14 +999,14 @@
       <c r="A11" t="s">
         <v>12</v>
       </c>
-      <c r="B11" t="s">
-        <v>112</v>
-      </c>
-      <c r="C11" t="s">
-        <v>112</v>
-      </c>
-      <c r="D11" t="s">
-        <v>112</v>
+      <c r="B11">
+        <v>45833.97</v>
+      </c>
+      <c r="C11">
+        <v>24801.47</v>
+      </c>
+      <c r="D11">
+        <v>17852.439999999999</v>
       </c>
       <c r="E11">
         <v>14424.51</v>
@@ -1034,14 +1022,14 @@
       <c r="A12" t="s">
         <v>13</v>
       </c>
-      <c r="B12" t="s">
-        <v>112</v>
-      </c>
-      <c r="C12" t="s">
-        <v>112</v>
-      </c>
-      <c r="D12" t="s">
-        <v>112</v>
+      <c r="B12">
+        <v>49657.2</v>
+      </c>
+      <c r="C12">
+        <v>26868.26</v>
+      </c>
+      <c r="D12">
+        <v>19340.14</v>
       </c>
       <c r="E12">
         <v>15626.55</v>
@@ -1057,14 +1045,14 @@
       <c r="A13" t="s">
         <v>14</v>
       </c>
-      <c r="B13" t="s">
-        <v>112</v>
-      </c>
-      <c r="C13" t="s">
-        <v>112</v>
-      </c>
-      <c r="D13" t="s">
-        <v>112</v>
+      <c r="B13">
+        <v>53473.54</v>
+      </c>
+      <c r="C13">
+        <v>28935.05</v>
+      </c>
+      <c r="D13">
+        <v>20827.849999999999</v>
       </c>
       <c r="E13">
         <v>16828.59</v>
@@ -1103,14 +1091,14 @@
       <c r="A15" t="s">
         <v>16</v>
       </c>
-      <c r="B15" t="s">
-        <v>112</v>
-      </c>
-      <c r="C15" t="s">
-        <v>112</v>
-      </c>
-      <c r="D15" t="s">
-        <v>112</v>
+      <c r="B15">
+        <v>61116.55</v>
+      </c>
+      <c r="C15">
+        <v>33068.620000000003</v>
+      </c>
+      <c r="D15">
+        <v>23803.25</v>
       </c>
       <c r="E15">
         <v>19232.68</v>
@@ -1126,14 +1114,14 @@
       <c r="A16" t="s">
         <v>17</v>
       </c>
-      <c r="B16" t="s">
-        <v>112</v>
-      </c>
-      <c r="C16" t="s">
-        <v>112</v>
-      </c>
-      <c r="D16" t="s">
-        <v>112</v>
+      <c r="B16">
+        <v>64936.33</v>
+      </c>
+      <c r="C16">
+        <v>35135.410000000003</v>
+      </c>
+      <c r="D16">
+        <v>25290.959999999999</v>
       </c>
       <c r="E16">
         <v>20434.72</v>
@@ -1149,14 +1137,14 @@
       <c r="A17" t="s">
         <v>18</v>
       </c>
-      <c r="B17" t="s">
-        <v>112</v>
-      </c>
-      <c r="C17" t="s">
-        <v>112</v>
-      </c>
-      <c r="D17" t="s">
-        <v>112</v>
+      <c r="B17">
+        <v>68756.12</v>
+      </c>
+      <c r="C17">
+        <v>37202.199999999997</v>
+      </c>
+      <c r="D17">
+        <v>26778.66</v>
       </c>
       <c r="E17">
         <v>21636.76</v>
@@ -1172,14 +1160,14 @@
       <c r="A18" t="s">
         <v>19</v>
       </c>
-      <c r="B18" t="s">
-        <v>112</v>
-      </c>
-      <c r="C18" t="s">
-        <v>112</v>
-      </c>
-      <c r="D18" t="s">
-        <v>112</v>
+      <c r="B18">
+        <v>72575.899999999994</v>
+      </c>
+      <c r="C18">
+        <v>39268.99</v>
+      </c>
+      <c r="D18">
+        <v>28266.36</v>
       </c>
       <c r="E18">
         <v>22838.799999999999</v>
@@ -1218,14 +1206,14 @@
       <c r="A20" t="s">
         <v>21</v>
       </c>
-      <c r="B20" t="s">
-        <v>112</v>
-      </c>
-      <c r="C20" t="s">
-        <v>112</v>
-      </c>
-      <c r="D20" t="s">
-        <v>112</v>
+      <c r="B20">
+        <v>80215.47</v>
+      </c>
+      <c r="C20">
+        <v>43402.57</v>
+      </c>
+      <c r="D20">
+        <v>31241.77</v>
       </c>
       <c r="E20">
         <v>25242.89</v>
@@ -1241,14 +1229,14 @@
       <c r="A21" t="s">
         <v>22</v>
       </c>
-      <c r="B21" t="s">
-        <v>112</v>
-      </c>
-      <c r="C21" t="s">
-        <v>112</v>
-      </c>
-      <c r="D21" t="s">
-        <v>112</v>
+      <c r="B21">
+        <v>84035.26</v>
+      </c>
+      <c r="C21">
+        <v>45469.36</v>
+      </c>
+      <c r="D21">
+        <v>32729.47</v>
       </c>
       <c r="E21">
         <v>26444.93</v>
@@ -1264,14 +1252,14 @@
       <c r="A22" t="s">
         <v>23</v>
       </c>
-      <c r="B22" t="s">
-        <v>112</v>
-      </c>
-      <c r="C22" t="s">
-        <v>112</v>
-      </c>
-      <c r="D22" t="s">
-        <v>112</v>
+      <c r="B22">
+        <v>87855.039999999994</v>
+      </c>
+      <c r="C22">
+        <v>47536.15</v>
+      </c>
+      <c r="D22">
+        <v>34217.18</v>
       </c>
       <c r="E22">
         <v>27646.97</v>
@@ -1287,14 +1275,14 @@
       <c r="A23" t="s">
         <v>24</v>
       </c>
-      <c r="B23" t="s">
-        <v>112</v>
-      </c>
-      <c r="C23" t="s">
-        <v>112</v>
-      </c>
-      <c r="D23" t="s">
-        <v>112</v>
+      <c r="B23">
+        <v>91674.82</v>
+      </c>
+      <c r="C23">
+        <v>49602.94</v>
+      </c>
+      <c r="D23">
+        <v>35704.879999999997</v>
       </c>
       <c r="E23">
         <v>28848.01</v>
@@ -1333,14 +1321,14 @@
       <c r="A25" t="s">
         <v>26</v>
       </c>
-      <c r="B25" t="s">
-        <v>112</v>
-      </c>
-      <c r="C25" t="s">
-        <v>112</v>
-      </c>
-      <c r="D25" t="s">
-        <v>112</v>
+      <c r="B25">
+        <v>99314.39</v>
+      </c>
+      <c r="C25">
+        <v>53736.51</v>
+      </c>
+      <c r="D25">
+        <v>38680.29</v>
       </c>
       <c r="E25">
         <v>31253.1</v>
@@ -1356,14 +1344,14 @@
       <c r="A26" t="s">
         <v>27</v>
       </c>
-      <c r="B26" t="s">
-        <v>112</v>
-      </c>
-      <c r="C26" t="s">
-        <v>112</v>
-      </c>
-      <c r="D26" t="s">
-        <v>112</v>
+      <c r="B26">
+        <v>103134.18</v>
+      </c>
+      <c r="C26">
+        <v>55803.3</v>
+      </c>
+      <c r="D26">
+        <v>40167.99</v>
       </c>
       <c r="E26">
         <v>32455.14</v>
@@ -1379,14 +1367,14 @@
       <c r="A27" t="s">
         <v>28</v>
       </c>
-      <c r="B27" t="s">
-        <v>112</v>
-      </c>
-      <c r="C27" t="s">
-        <v>112</v>
-      </c>
-      <c r="D27" t="s">
-        <v>112</v>
+      <c r="B27">
+        <v>106953.96</v>
+      </c>
+      <c r="C27">
+        <v>57870.09</v>
+      </c>
+      <c r="D27">
+        <v>41655.69</v>
       </c>
       <c r="E27">
         <v>33657.18</v>
@@ -1402,14 +1390,14 @@
       <c r="A28" t="s">
         <v>29</v>
       </c>
-      <c r="B28" t="s">
-        <v>112</v>
-      </c>
-      <c r="C28" t="s">
-        <v>112</v>
-      </c>
-      <c r="D28" t="s">
-        <v>112</v>
+      <c r="B28">
+        <v>110773.75</v>
+      </c>
+      <c r="C28">
+        <v>59936.88</v>
+      </c>
+      <c r="D28">
+        <v>43413.4</v>
       </c>
       <c r="E28">
         <v>34859.22</v>
@@ -1448,14 +1436,14 @@
       <c r="A30" t="s">
         <v>31</v>
       </c>
-      <c r="B30" t="s">
-        <v>112</v>
-      </c>
-      <c r="C30" t="s">
-        <v>112</v>
-      </c>
-      <c r="D30" t="s">
-        <v>112</v>
+      <c r="B30">
+        <v>118413.31</v>
+      </c>
+      <c r="C30">
+        <v>64070.46</v>
+      </c>
+      <c r="D30">
+        <v>46118.8</v>
       </c>
       <c r="E30">
         <v>37263.31</v>
@@ -1471,14 +1459,14 @@
       <c r="A31" t="s">
         <v>32</v>
       </c>
-      <c r="B31" t="s">
-        <v>112</v>
-      </c>
-      <c r="C31" t="s">
-        <v>112</v>
-      </c>
-      <c r="D31" t="s">
-        <v>112</v>
+      <c r="B31">
+        <v>122233.1</v>
+      </c>
+      <c r="C31">
+        <v>66137.25</v>
+      </c>
+      <c r="D31">
+        <v>47606.51</v>
       </c>
       <c r="E31">
         <v>38465.35</v>
@@ -1494,14 +1482,14 @@
       <c r="A32" t="s">
         <v>33</v>
       </c>
-      <c r="B32" t="s">
-        <v>112</v>
-      </c>
-      <c r="C32" t="s">
-        <v>112</v>
-      </c>
-      <c r="D32" t="s">
-        <v>112</v>
+      <c r="B32">
+        <v>126052.88</v>
+      </c>
+      <c r="C32">
+        <v>68204.039999999994</v>
+      </c>
+      <c r="D32">
+        <v>49094.21</v>
       </c>
       <c r="E32">
         <v>39667.39</v>
@@ -1517,14 +1505,14 @@
       <c r="A33" t="s">
         <v>34</v>
       </c>
-      <c r="B33" t="s">
-        <v>112</v>
-      </c>
-      <c r="C33" t="s">
-        <v>112</v>
-      </c>
-      <c r="D33" t="s">
-        <v>112</v>
+      <c r="B33">
+        <v>129872.67</v>
+      </c>
+      <c r="C33">
+        <v>70270.83</v>
+      </c>
+      <c r="D33">
+        <v>50581.91</v>
       </c>
       <c r="E33">
         <v>40869.440000000002</v>
@@ -1563,14 +1551,14 @@
       <c r="A35" t="s">
         <v>36</v>
       </c>
-      <c r="B35" t="s">
-        <v>112</v>
-      </c>
-      <c r="C35" t="s">
-        <v>112</v>
-      </c>
-      <c r="D35" t="s">
-        <v>112</v>
+      <c r="B35">
+        <v>137512.24</v>
+      </c>
+      <c r="C35">
+        <v>74404.399999999994</v>
+      </c>
+      <c r="D35">
+        <v>53557.32</v>
       </c>
       <c r="E35">
         <v>43273.52</v>
@@ -1586,14 +1574,14 @@
       <c r="A36" t="s">
         <v>37</v>
       </c>
-      <c r="B36" t="s">
-        <v>112</v>
-      </c>
-      <c r="C36" t="s">
-        <v>112</v>
-      </c>
-      <c r="D36" t="s">
-        <v>112</v>
+      <c r="B36">
+        <v>141332.01999999999</v>
+      </c>
+      <c r="C36">
+        <v>76471.19</v>
+      </c>
+      <c r="D36">
+        <v>55045.02</v>
       </c>
       <c r="E36">
         <v>44475.56</v>
@@ -1609,14 +1597,14 @@
       <c r="A37" t="s">
         <v>38</v>
       </c>
-      <c r="B37" t="s">
-        <v>112</v>
-      </c>
-      <c r="C37" t="s">
-        <v>112</v>
-      </c>
-      <c r="D37" t="s">
-        <v>112</v>
+      <c r="B37">
+        <v>145151.79999999999</v>
+      </c>
+      <c r="C37">
+        <v>78537.98</v>
+      </c>
+      <c r="D37">
+        <v>56532.72</v>
       </c>
       <c r="E37">
         <v>45667.6</v>
@@ -1632,14 +1620,14 @@
       <c r="A38" t="s">
         <v>39</v>
       </c>
-      <c r="B38" t="s">
-        <v>112</v>
-      </c>
-      <c r="C38" t="s">
-        <v>112</v>
-      </c>
-      <c r="D38" t="s">
-        <v>112</v>
+      <c r="B38">
+        <v>148971.59</v>
+      </c>
+      <c r="C38">
+        <v>80604.77</v>
+      </c>
+      <c r="D38">
+        <v>58020.43</v>
       </c>
       <c r="E38">
         <v>46879.65</v>
@@ -1678,14 +1666,14 @@
       <c r="A40" t="s">
         <v>41</v>
       </c>
-      <c r="B40" t="s">
-        <v>112</v>
-      </c>
-      <c r="C40" t="s">
-        <v>112</v>
-      </c>
-      <c r="D40" t="s">
-        <v>112</v>
+      <c r="B40">
+        <v>156611.16</v>
+      </c>
+      <c r="C40">
+        <v>84738.35</v>
+      </c>
+      <c r="D40">
+        <v>60995.83</v>
       </c>
       <c r="E40">
         <v>49283.73</v>
@@ -1701,14 +1689,14 @@
       <c r="A41" t="s">
         <v>42</v>
       </c>
-      <c r="B41" t="s">
-        <v>112</v>
-      </c>
-      <c r="C41" t="s">
-        <v>112</v>
-      </c>
-      <c r="D41" t="s">
-        <v>112</v>
+      <c r="B41">
+        <v>160430.94</v>
+      </c>
+      <c r="C41">
+        <v>86805.14</v>
+      </c>
+      <c r="D41">
+        <v>62483.54</v>
       </c>
       <c r="E41">
         <v>50485.77</v>
@@ -1724,14 +1712,14 @@
       <c r="A42" t="s">
         <v>43</v>
       </c>
-      <c r="B42" t="s">
-        <v>112</v>
-      </c>
-      <c r="C42" t="s">
-        <v>112</v>
-      </c>
-      <c r="D42" t="s">
-        <v>112</v>
+      <c r="B42">
+        <v>164250.73000000001</v>
+      </c>
+      <c r="C42">
+        <v>88871.93</v>
+      </c>
+      <c r="D42">
+        <v>63971.24</v>
       </c>
       <c r="E42">
         <v>51687.82</v>
@@ -1747,14 +1735,14 @@
       <c r="A43" t="s">
         <v>44</v>
       </c>
-      <c r="B43" t="s">
-        <v>112</v>
-      </c>
-      <c r="C43" t="s">
-        <v>112</v>
-      </c>
-      <c r="D43" t="s">
-        <v>112</v>
+      <c r="B43">
+        <v>168070.51</v>
+      </c>
+      <c r="C43">
+        <v>90938.72</v>
+      </c>
+      <c r="D43">
+        <v>65458.94</v>
       </c>
       <c r="E43">
         <v>52889.86</v>
@@ -1782,7 +1770,7 @@
       <c r="E44">
         <v>54091.9</v>
       </c>
-      <c r="F44" s="3">
+      <c r="F44" s="1">
         <v>41577.269999999997</v>
       </c>
       <c r="G44">
@@ -1793,14 +1781,14 @@
       <c r="A45" t="s">
         <v>46</v>
       </c>
-      <c r="B45" t="s">
-        <v>112</v>
-      </c>
-      <c r="C45" t="s">
-        <v>112</v>
-      </c>
-      <c r="D45" t="s">
-        <v>112</v>
+      <c r="B45">
+        <v>175710.07999999999</v>
+      </c>
+      <c r="C45">
+        <v>95072.29</v>
+      </c>
+      <c r="D45">
+        <v>68434.350000000006</v>
       </c>
       <c r="E45">
         <v>55293.94</v>
@@ -1816,14 +1804,14 @@
       <c r="A46" t="s">
         <v>47</v>
       </c>
-      <c r="B46" t="s">
-        <v>112</v>
-      </c>
-      <c r="C46" t="s">
-        <v>112</v>
-      </c>
-      <c r="D46" t="s">
-        <v>112</v>
+      <c r="B46">
+        <v>179529.86</v>
+      </c>
+      <c r="C46">
+        <v>97139.08</v>
+      </c>
+      <c r="D46">
+        <v>69922.05</v>
       </c>
       <c r="E46">
         <v>56495.98</v>
@@ -1839,14 +1827,14 @@
       <c r="A47" t="s">
         <v>48</v>
       </c>
-      <c r="B47" t="s">
-        <v>112</v>
-      </c>
-      <c r="C47" t="s">
-        <v>112</v>
-      </c>
-      <c r="D47" t="s">
-        <v>112</v>
+      <c r="B47">
+        <v>183349.65</v>
+      </c>
+      <c r="C47">
+        <v>99205.87</v>
+      </c>
+      <c r="D47">
+        <v>71409.759999999995</v>
       </c>
       <c r="E47">
         <v>57698.03</v>
@@ -1862,14 +1850,14 @@
       <c r="A48" t="s">
         <v>49</v>
       </c>
-      <c r="B48" t="s">
-        <v>112</v>
-      </c>
-      <c r="C48" t="s">
-        <v>112</v>
-      </c>
-      <c r="D48" t="s">
-        <v>112</v>
+      <c r="B48">
+        <v>187169.43</v>
+      </c>
+      <c r="C48">
+        <v>101272.66</v>
+      </c>
+      <c r="D48">
+        <v>72897.460000000006</v>
       </c>
       <c r="E48">
         <v>59800.07</v>
@@ -1908,14 +1896,14 @@
       <c r="A50" t="s">
         <v>51</v>
       </c>
-      <c r="B50" t="s">
-        <v>112</v>
-      </c>
-      <c r="C50" t="s">
-        <v>112</v>
-      </c>
-      <c r="D50" t="s">
-        <v>112</v>
+      <c r="B50">
+        <v>194809</v>
+      </c>
+      <c r="C50">
+        <v>105406.24</v>
+      </c>
+      <c r="D50">
+        <v>75872.87</v>
       </c>
       <c r="E50">
         <v>61304.15</v>
@@ -1931,14 +1919,14 @@
       <c r="A51" t="s">
         <v>52</v>
       </c>
-      <c r="B51" t="s">
-        <v>112</v>
-      </c>
-      <c r="C51" t="s">
-        <v>112</v>
-      </c>
-      <c r="D51" t="s">
-        <v>112</v>
+      <c r="B51">
+        <v>198628.79</v>
+      </c>
+      <c r="C51">
+        <v>107473.03</v>
+      </c>
+      <c r="D51">
+        <v>77360.570000000007</v>
       </c>
       <c r="E51">
         <v>62506.2</v>
@@ -1954,14 +1942,14 @@
       <c r="A52" t="s">
         <v>53</v>
       </c>
-      <c r="B52" t="s">
-        <v>112</v>
-      </c>
-      <c r="C52" t="s">
-        <v>112</v>
-      </c>
-      <c r="D52" t="s">
-        <v>112</v>
+      <c r="B52">
+        <v>202448.57</v>
+      </c>
+      <c r="C52">
+        <v>109539.82</v>
+      </c>
+      <c r="D52">
+        <v>78848.27</v>
       </c>
       <c r="E52">
         <v>63708.24</v>
@@ -1977,14 +1965,14 @@
       <c r="A53" t="s">
         <v>54</v>
       </c>
-      <c r="B53" t="s">
-        <v>112</v>
-      </c>
-      <c r="C53" t="s">
-        <v>112</v>
-      </c>
-      <c r="D53" t="s">
-        <v>112</v>
+      <c r="B53">
+        <v>206268.35</v>
+      </c>
+      <c r="C53">
+        <v>111606.61</v>
+      </c>
+      <c r="D53">
+        <v>80335.98</v>
       </c>
       <c r="E53">
         <v>64910.28</v>
@@ -2023,14 +2011,14 @@
       <c r="A55" t="s">
         <v>56</v>
       </c>
-      <c r="B55" t="s">
-        <v>112</v>
-      </c>
-      <c r="C55" t="s">
-        <v>112</v>
-      </c>
-      <c r="D55" t="s">
-        <v>112</v>
+      <c r="B55">
+        <v>213907.92</v>
+      </c>
+      <c r="C55">
+        <v>115740.18</v>
+      </c>
+      <c r="D55">
+        <v>83311.38</v>
       </c>
       <c r="E55">
         <v>67314.36</v>
@@ -2046,14 +2034,14 @@
       <c r="A56" t="s">
         <v>57</v>
       </c>
-      <c r="B56" t="s">
-        <v>112</v>
-      </c>
-      <c r="C56" t="s">
-        <v>112</v>
-      </c>
-      <c r="D56" t="s">
-        <v>112</v>
+      <c r="B56">
+        <v>217727.71</v>
+      </c>
+      <c r="C56">
+        <v>117806.97</v>
+      </c>
+      <c r="D56">
+        <v>84799.09</v>
       </c>
       <c r="E56">
         <v>68516.41</v>
@@ -2069,14 +2057,14 @@
       <c r="A57" t="s">
         <v>58</v>
       </c>
-      <c r="B57" t="s">
-        <v>112</v>
-      </c>
-      <c r="C57" t="s">
-        <v>112</v>
-      </c>
-      <c r="D57" t="s">
-        <v>112</v>
+      <c r="B57">
+        <v>221547.49</v>
+      </c>
+      <c r="C57">
+        <v>119873.76</v>
+      </c>
+      <c r="D57">
+        <v>86286.79</v>
       </c>
       <c r="E57">
         <v>69718.45</v>
@@ -2092,14 +2080,14 @@
       <c r="A58" t="s">
         <v>59</v>
       </c>
-      <c r="B58" t="s">
-        <v>112</v>
-      </c>
-      <c r="C58" t="s">
-        <v>112</v>
-      </c>
-      <c r="D58" t="s">
-        <v>112</v>
+      <c r="B58">
+        <v>225367.28</v>
+      </c>
+      <c r="C58">
+        <v>121940.55</v>
+      </c>
+      <c r="D58">
+        <v>87774.49</v>
       </c>
       <c r="E58">
         <v>70920.490000000005</v>
@@ -2138,14 +2126,14 @@
       <c r="A60" t="s">
         <v>61</v>
       </c>
-      <c r="B60" t="s">
-        <v>112</v>
-      </c>
-      <c r="C60" t="s">
-        <v>112</v>
-      </c>
-      <c r="D60" t="s">
-        <v>112</v>
+      <c r="B60">
+        <v>233006.84</v>
+      </c>
+      <c r="C60">
+        <v>126074.13</v>
+      </c>
+      <c r="D60">
+        <v>90749.9</v>
       </c>
       <c r="E60">
         <v>73324.58</v>
@@ -2161,14 +2149,14 @@
       <c r="A61" t="s">
         <v>62</v>
       </c>
-      <c r="B61" t="s">
-        <v>112</v>
-      </c>
-      <c r="C61" t="s">
-        <v>112</v>
-      </c>
-      <c r="D61" t="s">
-        <v>112</v>
+      <c r="B61">
+        <v>236826.63</v>
+      </c>
+      <c r="C61">
+        <v>128140.92</v>
+      </c>
+      <c r="D61">
+        <v>92237.6</v>
       </c>
       <c r="E61">
         <v>74526.62</v>
@@ -2184,14 +2172,14 @@
       <c r="A62" t="s">
         <v>63</v>
       </c>
-      <c r="B62" t="s">
-        <v>112</v>
-      </c>
-      <c r="C62" t="s">
-        <v>112</v>
-      </c>
-      <c r="D62" t="s">
-        <v>112</v>
+      <c r="B62">
+        <v>240646.41</v>
+      </c>
+      <c r="C62">
+        <v>130207.71</v>
+      </c>
+      <c r="D62">
+        <v>93725.31</v>
       </c>
       <c r="E62">
         <v>75728.66</v>
@@ -2207,14 +2195,14 @@
       <c r="A63" t="s">
         <v>64</v>
       </c>
-      <c r="B63" t="s">
-        <v>112</v>
-      </c>
-      <c r="C63" t="s">
-        <v>112</v>
-      </c>
-      <c r="D63" t="s">
-        <v>112</v>
+      <c r="B63">
+        <v>244466.2</v>
+      </c>
+      <c r="C63">
+        <v>132274.5</v>
+      </c>
+      <c r="D63">
+        <v>95213.01</v>
       </c>
       <c r="E63">
         <v>76930.7</v>
@@ -2253,14 +2241,14 @@
       <c r="A65" t="s">
         <v>66</v>
       </c>
-      <c r="B65" t="s">
-        <v>112</v>
-      </c>
-      <c r="C65" t="s">
-        <v>112</v>
-      </c>
-      <c r="D65" t="s">
-        <v>112</v>
+      <c r="B65">
+        <v>252105.77</v>
+      </c>
+      <c r="C65">
+        <v>136408.07</v>
+      </c>
+      <c r="D65">
+        <v>98188.42</v>
       </c>
       <c r="E65">
         <v>79334.789999999994</v>
@@ -2276,14 +2264,14 @@
       <c r="A66" t="s">
         <v>67</v>
       </c>
-      <c r="B66" t="s">
-        <v>112</v>
-      </c>
-      <c r="C66" t="s">
-        <v>112</v>
-      </c>
-      <c r="D66" t="s">
-        <v>112</v>
+      <c r="B66">
+        <v>255925.55</v>
+      </c>
+      <c r="C66">
+        <v>138474.85999999999</v>
+      </c>
+      <c r="D66">
+        <v>99676.12</v>
       </c>
       <c r="E66">
         <v>80536.83</v>
@@ -2299,14 +2287,14 @@
       <c r="A67" t="s">
         <v>68</v>
       </c>
-      <c r="B67" t="s">
-        <v>112</v>
-      </c>
-      <c r="C67" t="s">
-        <v>112</v>
-      </c>
-      <c r="D67" t="s">
-        <v>112</v>
+      <c r="B67">
+        <v>259745.33</v>
+      </c>
+      <c r="C67">
+        <v>140541.65</v>
+      </c>
+      <c r="D67">
+        <v>101163.82</v>
       </c>
       <c r="E67">
         <v>81738.87</v>
@@ -2322,14 +2310,14 @@
       <c r="A68" t="s">
         <v>69</v>
       </c>
-      <c r="B68" t="s">
-        <v>112</v>
-      </c>
-      <c r="C68" t="s">
-        <v>112</v>
-      </c>
-      <c r="D68" t="s">
-        <v>112</v>
+      <c r="B68">
+        <v>263565.12</v>
+      </c>
+      <c r="C68">
+        <v>142608.44</v>
+      </c>
+      <c r="D68">
+        <v>102651.53</v>
       </c>
       <c r="E68">
         <v>82940.91</v>
@@ -2345,14 +2333,14 @@
       <c r="A69" t="s">
         <v>70</v>
       </c>
-      <c r="B69" t="s">
-        <v>112</v>
-      </c>
-      <c r="C69" t="s">
-        <v>112</v>
-      </c>
-      <c r="D69" t="s">
-        <v>112</v>
+      <c r="B69">
+        <v>267384.90000000002</v>
+      </c>
+      <c r="C69">
+        <v>144675.23000000001</v>
+      </c>
+      <c r="D69">
+        <v>104139.23</v>
       </c>
       <c r="E69">
         <v>84142.96</v>
@@ -2368,14 +2356,14 @@
       <c r="A70" t="s">
         <v>71</v>
       </c>
-      <c r="B70" t="s">
-        <v>112</v>
-      </c>
-      <c r="C70" t="s">
-        <v>112</v>
-      </c>
-      <c r="D70" t="s">
-        <v>112</v>
+      <c r="B70">
+        <v>271204.69</v>
+      </c>
+      <c r="C70">
+        <v>146742.01999999999</v>
+      </c>
+      <c r="D70">
+        <v>105626.93</v>
       </c>
       <c r="E70">
         <v>85345</v>
@@ -2391,14 +2379,14 @@
       <c r="A71" t="s">
         <v>72</v>
       </c>
-      <c r="B71" t="s">
-        <v>112</v>
-      </c>
-      <c r="C71" t="s">
-        <v>112</v>
-      </c>
-      <c r="D71" t="s">
-        <v>112</v>
+      <c r="B71">
+        <v>275024.46999999997</v>
+      </c>
+      <c r="C71">
+        <v>148808.81</v>
+      </c>
+      <c r="D71">
+        <v>107114.64</v>
       </c>
       <c r="E71">
         <v>86547.04</v>
@@ -2414,14 +2402,14 @@
       <c r="A72" t="s">
         <v>73</v>
       </c>
-      <c r="B72" t="s">
-        <v>112</v>
-      </c>
-      <c r="C72" t="s">
-        <v>112</v>
-      </c>
-      <c r="D72" t="s">
-        <v>112</v>
+      <c r="B72">
+        <v>278844.26</v>
+      </c>
+      <c r="C72">
+        <v>150875.6</v>
+      </c>
+      <c r="D72">
+        <v>108602.34</v>
       </c>
       <c r="E72">
         <v>87749.08</v>
@@ -2437,14 +2425,14 @@
       <c r="A73" t="s">
         <v>74</v>
       </c>
-      <c r="B73" t="s">
-        <v>112</v>
-      </c>
-      <c r="C73" t="s">
-        <v>112</v>
-      </c>
-      <c r="D73" t="s">
-        <v>112</v>
+      <c r="B73">
+        <v>282664.03999999998</v>
+      </c>
+      <c r="C73">
+        <v>152942.39000000001</v>
+      </c>
+      <c r="D73">
+        <v>110090.04</v>
       </c>
       <c r="E73">
         <v>88951.12</v>
@@ -2460,14 +2448,14 @@
       <c r="A74" t="s">
         <v>75</v>
       </c>
-      <c r="B74" t="s">
-        <v>112</v>
-      </c>
-      <c r="C74" t="s">
-        <v>112</v>
-      </c>
-      <c r="D74" t="s">
-        <v>112</v>
+      <c r="B74">
+        <v>286483.82</v>
+      </c>
+      <c r="C74">
+        <v>155009.18</v>
+      </c>
+      <c r="D74">
+        <v>111577.75</v>
       </c>
       <c r="E74">
         <v>90153.17</v>
@@ -2483,14 +2471,14 @@
       <c r="A75" t="s">
         <v>76</v>
       </c>
-      <c r="B75" t="s">
-        <v>112</v>
-      </c>
-      <c r="C75" t="s">
-        <v>112</v>
-      </c>
-      <c r="D75" t="s">
-        <v>112</v>
+      <c r="B75">
+        <v>290303.61</v>
+      </c>
+      <c r="C75">
+        <v>157075.96</v>
+      </c>
+      <c r="D75">
+        <v>113065.45</v>
       </c>
       <c r="E75">
         <v>91355.21</v>
@@ -2506,14 +2494,14 @@
       <c r="A76" t="s">
         <v>77</v>
       </c>
-      <c r="B76" t="s">
-        <v>112</v>
-      </c>
-      <c r="C76" t="s">
-        <v>112</v>
-      </c>
-      <c r="D76" t="s">
-        <v>112</v>
+      <c r="B76">
+        <v>294123.39</v>
+      </c>
+      <c r="C76">
+        <v>159142.75</v>
+      </c>
+      <c r="D76">
+        <v>114553.15</v>
       </c>
       <c r="E76">
         <v>92557.25</v>
@@ -2529,14 +2517,14 @@
       <c r="A77" t="s">
         <v>78</v>
       </c>
-      <c r="B77" t="s">
-        <v>112</v>
-      </c>
-      <c r="C77" t="s">
-        <v>112</v>
-      </c>
-      <c r="D77" t="s">
-        <v>112</v>
+      <c r="B77">
+        <v>297943.18</v>
+      </c>
+      <c r="C77">
+        <v>161209.54</v>
+      </c>
+      <c r="D77">
+        <v>116040.86</v>
       </c>
       <c r="E77">
         <v>93759.29</v>
@@ -2552,14 +2540,14 @@
       <c r="A78" t="s">
         <v>79</v>
       </c>
-      <c r="B78" t="s">
-        <v>112</v>
-      </c>
-      <c r="C78" t="s">
-        <v>112</v>
-      </c>
-      <c r="D78" t="s">
-        <v>112</v>
+      <c r="B78">
+        <v>301762.96000000002</v>
+      </c>
+      <c r="C78">
+        <v>163276.32999999999</v>
+      </c>
+      <c r="D78">
+        <v>117528.56</v>
       </c>
       <c r="E78">
         <v>94961.34</v>
@@ -2575,14 +2563,14 @@
       <c r="A79" t="s">
         <v>80</v>
       </c>
-      <c r="B79" t="s">
-        <v>112</v>
-      </c>
-      <c r="C79" t="s">
-        <v>112</v>
-      </c>
-      <c r="D79" t="s">
-        <v>112</v>
+      <c r="B79">
+        <v>305582.75</v>
+      </c>
+      <c r="C79">
+        <v>165343.12</v>
+      </c>
+      <c r="D79">
+        <v>119016.26</v>
       </c>
       <c r="E79">
         <v>96163.38</v>
@@ -2598,14 +2586,14 @@
       <c r="A80" t="s">
         <v>81</v>
       </c>
-      <c r="B80" t="s">
-        <v>112</v>
-      </c>
-      <c r="C80" t="s">
-        <v>112</v>
-      </c>
-      <c r="D80" t="s">
-        <v>112</v>
+      <c r="B80">
+        <v>309402.53000000003</v>
+      </c>
+      <c r="C80">
+        <v>167409.91</v>
+      </c>
+      <c r="D80">
+        <v>120503.97</v>
       </c>
       <c r="E80">
         <v>97365.42</v>
@@ -2621,14 +2609,14 @@
       <c r="A81" t="s">
         <v>82</v>
       </c>
-      <c r="B81" t="s">
-        <v>112</v>
-      </c>
-      <c r="C81" t="s">
-        <v>112</v>
-      </c>
-      <c r="D81" t="s">
-        <v>112</v>
+      <c r="B81">
+        <v>313222.32</v>
+      </c>
+      <c r="C81">
+        <v>169476.7</v>
+      </c>
+      <c r="D81">
+        <v>121991.67</v>
       </c>
       <c r="E81">
         <v>98567.46</v>
@@ -2644,14 +2632,14 @@
       <c r="A82" t="s">
         <v>83</v>
       </c>
-      <c r="B82" t="s">
-        <v>112</v>
-      </c>
-      <c r="C82" t="s">
-        <v>112</v>
-      </c>
-      <c r="D82" t="s">
-        <v>112</v>
+      <c r="B82">
+        <v>317042.09999999998</v>
+      </c>
+      <c r="C82">
+        <v>171543.49</v>
+      </c>
+      <c r="D82">
+        <v>123479.37</v>
       </c>
       <c r="E82">
         <v>99769.5</v>
@@ -2667,14 +2655,14 @@
       <c r="A83" t="s">
         <v>84</v>
       </c>
-      <c r="B83" t="s">
-        <v>112</v>
-      </c>
-      <c r="C83" t="s">
-        <v>112</v>
-      </c>
-      <c r="D83" t="s">
-        <v>112</v>
+      <c r="B83">
+        <v>320861.88</v>
+      </c>
+      <c r="C83">
+        <v>173610.28</v>
+      </c>
+      <c r="D83">
+        <v>124967.08</v>
       </c>
       <c r="E83">
         <v>100971.55</v>
@@ -2690,14 +2678,14 @@
       <c r="A84" t="s">
         <v>85</v>
       </c>
-      <c r="B84" t="s">
-        <v>112</v>
-      </c>
-      <c r="C84" t="s">
-        <v>112</v>
-      </c>
-      <c r="D84" t="s">
-        <v>112</v>
+      <c r="B84">
+        <v>324681.67</v>
+      </c>
+      <c r="C84">
+        <v>175677.07</v>
+      </c>
+      <c r="D84">
+        <v>126454.78</v>
       </c>
       <c r="E84">
         <v>102173.59</v>
@@ -2713,14 +2701,14 @@
       <c r="A85" t="s">
         <v>86</v>
       </c>
-      <c r="B85" t="s">
-        <v>112</v>
-      </c>
-      <c r="C85" t="s">
-        <v>112</v>
-      </c>
-      <c r="D85" t="s">
-        <v>112</v>
+      <c r="B85">
+        <v>328501.45</v>
+      </c>
+      <c r="C85">
+        <v>177743.85</v>
+      </c>
+      <c r="D85">
+        <v>127942.48</v>
       </c>
       <c r="E85">
         <v>103375.63</v>
@@ -2736,14 +2724,14 @@
       <c r="A86" t="s">
         <v>87</v>
       </c>
-      <c r="B86" t="s">
-        <v>112</v>
-      </c>
-      <c r="C86" t="s">
-        <v>112</v>
-      </c>
-      <c r="D86" t="s">
-        <v>112</v>
+      <c r="B86">
+        <v>332321.24</v>
+      </c>
+      <c r="C86">
+        <v>179810.64</v>
+      </c>
+      <c r="D86">
+        <v>129430.19</v>
       </c>
       <c r="E86">
         <v>104577.67</v>
@@ -2759,14 +2747,14 @@
       <c r="A87" t="s">
         <v>88</v>
       </c>
-      <c r="B87" t="s">
-        <v>112</v>
-      </c>
-      <c r="C87" t="s">
-        <v>112</v>
-      </c>
-      <c r="D87" t="s">
-        <v>112</v>
+      <c r="B87">
+        <v>336141.02</v>
+      </c>
+      <c r="C87">
+        <v>181877.43</v>
+      </c>
+      <c r="D87">
+        <v>130917.89</v>
       </c>
       <c r="E87">
         <v>105779.72</v>
@@ -2782,14 +2770,14 @@
       <c r="A88" t="s">
         <v>89</v>
       </c>
-      <c r="B88" t="s">
-        <v>112</v>
-      </c>
-      <c r="C88" t="s">
-        <v>112</v>
-      </c>
-      <c r="D88" t="s">
-        <v>112</v>
+      <c r="B88">
+        <v>339960.81</v>
+      </c>
+      <c r="C88">
+        <v>183944.22</v>
+      </c>
+      <c r="D88">
+        <v>132405.59</v>
       </c>
       <c r="E88">
         <v>106981.75999999999</v>
@@ -2805,14 +2793,14 @@
       <c r="A89" t="s">
         <v>90</v>
       </c>
-      <c r="B89" t="s">
-        <v>112</v>
-      </c>
-      <c r="C89" t="s">
-        <v>112</v>
-      </c>
-      <c r="D89" t="s">
-        <v>112</v>
+      <c r="B89">
+        <v>343780.59</v>
+      </c>
+      <c r="C89">
+        <v>186011.01</v>
+      </c>
+      <c r="D89">
+        <v>133893.29999999999</v>
       </c>
       <c r="E89">
         <v>108183.8</v>
@@ -2828,14 +2816,14 @@
       <c r="A90" t="s">
         <v>91</v>
       </c>
-      <c r="B90" t="s">
-        <v>112</v>
-      </c>
-      <c r="C90" t="s">
-        <v>112</v>
-      </c>
-      <c r="D90" t="s">
-        <v>112</v>
+      <c r="B90">
+        <v>347600.37</v>
+      </c>
+      <c r="C90">
+        <v>188077.8</v>
+      </c>
+      <c r="D90">
+        <v>135381</v>
       </c>
       <c r="E90">
         <v>109385.84</v>
@@ -2851,14 +2839,14 @@
       <c r="A91" t="s">
         <v>92</v>
       </c>
-      <c r="B91" t="s">
-        <v>112</v>
-      </c>
-      <c r="C91" t="s">
-        <v>112</v>
-      </c>
-      <c r="D91" t="s">
-        <v>112</v>
+      <c r="B91">
+        <v>351420.15999999997</v>
+      </c>
+      <c r="C91">
+        <v>190144.59</v>
+      </c>
+      <c r="D91">
+        <v>136868.70000000001</v>
       </c>
       <c r="E91">
         <v>110587.88</v>
@@ -2874,14 +2862,14 @@
       <c r="A92" t="s">
         <v>93</v>
       </c>
-      <c r="B92" t="s">
-        <v>112</v>
-      </c>
-      <c r="C92" t="s">
-        <v>112</v>
-      </c>
-      <c r="D92" t="s">
-        <v>112</v>
+      <c r="B92">
+        <v>355239.94</v>
+      </c>
+      <c r="C92">
+        <v>192211.38</v>
+      </c>
+      <c r="D92">
+        <v>138356.41</v>
       </c>
       <c r="E92">
         <v>111789.93</v>
@@ -2897,14 +2885,14 @@
       <c r="A93" t="s">
         <v>94</v>
       </c>
-      <c r="B93" t="s">
-        <v>112</v>
-      </c>
-      <c r="C93" t="s">
-        <v>112</v>
-      </c>
-      <c r="D93" t="s">
-        <v>112</v>
+      <c r="B93">
+        <v>359059.73</v>
+      </c>
+      <c r="C93">
+        <v>194278.17</v>
+      </c>
+      <c r="D93">
+        <v>139844.10999999999</v>
       </c>
       <c r="E93">
         <v>112991.97</v>
@@ -2920,14 +2908,14 @@
       <c r="A94" t="s">
         <v>95</v>
       </c>
-      <c r="B94" t="s">
-        <v>112</v>
-      </c>
-      <c r="C94" t="s">
-        <v>112</v>
-      </c>
-      <c r="D94" t="s">
-        <v>112</v>
+      <c r="B94">
+        <v>362879.51</v>
+      </c>
+      <c r="C94">
+        <v>196344.95999999999</v>
+      </c>
+      <c r="D94">
+        <v>141331.81</v>
       </c>
       <c r="E94">
         <v>114194.01</v>
@@ -2943,14 +2931,14 @@
       <c r="A95" t="s">
         <v>96</v>
       </c>
-      <c r="B95" t="s">
-        <v>112</v>
-      </c>
-      <c r="C95" t="s">
-        <v>112</v>
-      </c>
-      <c r="D95" t="s">
-        <v>112</v>
+      <c r="B95">
+        <v>366699.3</v>
+      </c>
+      <c r="C95">
+        <v>198411.74</v>
+      </c>
+      <c r="D95">
+        <v>142819.51999999999</v>
       </c>
       <c r="E95">
         <v>115396.05</v>
@@ -2966,14 +2954,14 @@
       <c r="A96" t="s">
         <v>97</v>
       </c>
-      <c r="B96" t="s">
-        <v>112</v>
-      </c>
-      <c r="C96" t="s">
-        <v>112</v>
-      </c>
-      <c r="D96" t="s">
-        <v>112</v>
+      <c r="B96">
+        <v>370519.08</v>
+      </c>
+      <c r="C96">
+        <v>200478.53</v>
+      </c>
+      <c r="D96">
+        <v>144307.22</v>
       </c>
       <c r="E96">
         <v>116598.1</v>
@@ -2989,14 +2977,14 @@
       <c r="A97" t="s">
         <v>98</v>
       </c>
-      <c r="B97" t="s">
-        <v>112</v>
-      </c>
-      <c r="C97" t="s">
-        <v>112</v>
-      </c>
-      <c r="D97" t="s">
-        <v>112</v>
+      <c r="B97">
+        <v>374338.86</v>
+      </c>
+      <c r="C97">
+        <v>202545.32</v>
+      </c>
+      <c r="D97">
+        <v>145794.92000000001</v>
       </c>
       <c r="E97">
         <v>117800.14</v>
@@ -3012,14 +3000,14 @@
       <c r="A98" t="s">
         <v>99</v>
       </c>
-      <c r="B98" t="s">
-        <v>112</v>
-      </c>
-      <c r="C98" t="s">
-        <v>112</v>
-      </c>
-      <c r="D98" t="s">
-        <v>112</v>
+      <c r="B98">
+        <v>378158.65</v>
+      </c>
+      <c r="C98">
+        <v>204612.11</v>
+      </c>
+      <c r="D98">
+        <v>147282.63</v>
       </c>
       <c r="E98">
         <v>119002.18</v>
@@ -3035,14 +3023,14 @@
       <c r="A99" t="s">
         <v>100</v>
       </c>
-      <c r="B99" t="s">
-        <v>112</v>
-      </c>
-      <c r="C99" t="s">
-        <v>112</v>
-      </c>
-      <c r="D99" t="s">
-        <v>112</v>
+      <c r="B99">
+        <v>381978.43</v>
+      </c>
+      <c r="C99">
+        <v>206678.9</v>
+      </c>
+      <c r="D99">
+        <v>148770.32999999999</v>
       </c>
       <c r="E99">
         <v>120204.22</v>
@@ -3058,14 +3046,14 @@
       <c r="A100" t="s">
         <v>101</v>
       </c>
-      <c r="B100" t="s">
-        <v>112</v>
-      </c>
-      <c r="C100" t="s">
-        <v>112</v>
-      </c>
-      <c r="D100" t="s">
-        <v>112</v>
+      <c r="B100">
+        <v>401077.35</v>
+      </c>
+      <c r="C100">
+        <v>217012.85</v>
+      </c>
+      <c r="D100">
+        <v>156208.84</v>
       </c>
       <c r="E100">
         <v>126214.43</v>
@@ -3081,14 +3069,14 @@
       <c r="A101" t="s">
         <v>102</v>
       </c>
-      <c r="B101" t="s">
-        <v>112</v>
-      </c>
-      <c r="C101" t="s">
-        <v>112</v>
-      </c>
-      <c r="D101" t="s">
-        <v>112</v>
+      <c r="B101">
+        <v>420176.28</v>
+      </c>
+      <c r="C101">
+        <v>227346.79</v>
+      </c>
+      <c r="D101">
+        <v>163647.35999999999</v>
       </c>
       <c r="E101">
         <v>132224.64000000001</v>
@@ -3104,14 +3092,14 @@
       <c r="A102" t="s">
         <v>103</v>
       </c>
-      <c r="B102" t="s">
-        <v>112</v>
-      </c>
-      <c r="C102" t="s">
-        <v>112</v>
-      </c>
-      <c r="D102" t="s">
-        <v>112</v>
+      <c r="B102">
+        <v>439275.2</v>
+      </c>
+      <c r="C102">
+        <v>237680.74</v>
+      </c>
+      <c r="D102">
+        <v>171085.88</v>
       </c>
       <c r="E102">
         <v>138234.85999999999</v>
@@ -3127,14 +3115,14 @@
       <c r="A103" t="s">
         <v>104</v>
       </c>
-      <c r="B103" t="s">
-        <v>112</v>
-      </c>
-      <c r="C103" t="s">
-        <v>112</v>
-      </c>
-      <c r="D103" t="s">
-        <v>112</v>
+      <c r="B103">
+        <v>458374.12</v>
+      </c>
+      <c r="C103">
+        <v>248014.68</v>
+      </c>
+      <c r="D103">
+        <v>178524.39</v>
       </c>
       <c r="E103">
         <v>144245.07</v>
@@ -3150,14 +3138,14 @@
       <c r="A104" t="s">
         <v>105</v>
       </c>
-      <c r="B104" t="s">
-        <v>112</v>
-      </c>
-      <c r="C104" t="s">
-        <v>112</v>
-      </c>
-      <c r="D104" t="s">
-        <v>112</v>
+      <c r="B104">
+        <v>477473.04</v>
+      </c>
+      <c r="C104">
+        <v>258348.63</v>
+      </c>
+      <c r="D104">
+        <v>15962.91</v>
       </c>
       <c r="E104">
         <v>150255.28</v>
@@ -3173,14 +3161,14 @@
       <c r="A105" t="s">
         <v>106</v>
       </c>
-      <c r="B105" t="s">
-        <v>112</v>
-      </c>
-      <c r="C105" t="s">
-        <v>112</v>
-      </c>
-      <c r="D105" t="s">
-        <v>112</v>
+      <c r="B105">
+        <v>496571.96</v>
+      </c>
+      <c r="C105">
+        <v>268682.57</v>
+      </c>
+      <c r="D105">
+        <v>193401.43</v>
       </c>
       <c r="E105">
         <v>156265.49</v>
@@ -3196,14 +3184,14 @@
       <c r="A106" t="s">
         <v>107</v>
       </c>
-      <c r="B106" t="s">
-        <v>112</v>
-      </c>
-      <c r="C106" t="s">
-        <v>112</v>
-      </c>
-      <c r="D106" t="s">
-        <v>112</v>
+      <c r="B106">
+        <v>515670.88</v>
+      </c>
+      <c r="C106">
+        <v>279016.52</v>
+      </c>
+      <c r="D106">
+        <v>200839.94</v>
       </c>
       <c r="E106">
         <v>162275.70000000001</v>
@@ -3219,14 +3207,14 @@
       <c r="A107" t="s">
         <v>108</v>
       </c>
-      <c r="B107" t="s">
-        <v>112</v>
-      </c>
-      <c r="C107" t="s">
-        <v>112</v>
-      </c>
-      <c r="D107" t="s">
-        <v>112</v>
+      <c r="B107">
+        <v>534769.81000000006</v>
+      </c>
+      <c r="C107">
+        <v>289350.46000000002</v>
+      </c>
+      <c r="D107">
+        <v>208278.46</v>
       </c>
       <c r="E107">
         <v>168285.91</v>
@@ -3242,14 +3230,14 @@
       <c r="A108" t="s">
         <v>109</v>
       </c>
-      <c r="B108" t="s">
-        <v>112</v>
-      </c>
-      <c r="C108" t="s">
-        <v>112</v>
-      </c>
-      <c r="D108" t="s">
-        <v>112</v>
+      <c r="B108">
+        <v>553868.73</v>
+      </c>
+      <c r="C108">
+        <v>299684.40999999997</v>
+      </c>
+      <c r="D108">
+        <v>215716.98</v>
       </c>
       <c r="E108">
         <v>174296.12</v>
@@ -3265,14 +3253,14 @@
       <c r="A109" t="s">
         <v>110</v>
       </c>
-      <c r="B109" t="s">
-        <v>112</v>
-      </c>
-      <c r="C109" t="s">
-        <v>112</v>
-      </c>
-      <c r="D109" t="s">
-        <v>112</v>
+      <c r="B109">
+        <v>572967.65</v>
+      </c>
+      <c r="C109">
+        <v>310018.34999999998</v>
+      </c>
+      <c r="D109">
+        <v>223155.49</v>
       </c>
       <c r="E109">
         <v>180306.33</v>

</xml_diff>